<commit_message>
#251226 fix: fixed global settings
</commit_message>
<xml_diff>
--- a/files/tufe.xlsx
+++ b/files/tufe.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\koray.zorlu\projects\arierp\arierp_backend\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D2EC103-466B-4C11-B7A2-F838D1FE7F5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FC00C63-4BE4-4D95-AB84-220F143CF39E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2120" yWindow="2120" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="255">
   <si>
     <t>Dönem</t>
   </si>
@@ -787,6 +787,9 @@
   </si>
   <si>
     <t xml:space="preserve">01-2005 </t>
+  </si>
+  <si>
+    <t>Gözlem Değeri</t>
   </si>
 </sst>
 </file>
@@ -822,10 +825,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1106,15 +1110,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C252"/>
+  <dimension ref="A1:D252"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.81640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="12.54296875" style="2" customWidth="1"/>
     <col min="3" max="3" width="14.08984375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1124,8 +1129,11 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D1" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1135,8 +1143,11 @@
       <c r="C2" s="2">
         <v>0.87</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D2" s="3">
+        <v>3482.96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1146,8 +1157,11 @@
       <c r="C3" s="2">
         <v>2.5499999999999998</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D3" s="3">
+        <v>3453.09</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -1157,8 +1171,11 @@
       <c r="C4" s="2">
         <v>3.23</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D4" s="3">
+        <v>3367.22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -1168,8 +1185,11 @@
       <c r="C5" s="2">
         <v>2.04</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D5" s="3">
+        <v>3261.72</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
@@ -1179,8 +1199,11 @@
       <c r="C6" s="2">
         <v>2.06</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D6" s="3">
+        <v>3196.66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -1190,8 +1213,11 @@
       <c r="C7" s="2">
         <v>1.37</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D7" s="3">
+        <v>3132.17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
@@ -1201,8 +1227,11 @@
       <c r="C8" s="2">
         <v>1.53</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D8" s="3">
+        <v>3089.74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -1212,8 +1241,11 @@
       <c r="C9" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D9" s="3">
+        <v>3043.23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -1223,8 +1255,11 @@
       <c r="C10" s="2">
         <v>2.46</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D10" s="3">
+        <v>2954.69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>12</v>
       </c>
@@ -1234,8 +1269,11 @@
       <c r="C11" s="2">
         <v>2.27</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D11" s="3">
+        <v>2883.75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>13</v>
       </c>
@@ -1245,8 +1283,11 @@
       <c r="C12" s="2">
         <v>5.03</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D12" s="3">
+        <v>2819.65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>14</v>
       </c>
@@ -1256,8 +1297,11 @@
       <c r="C13" s="2">
         <v>1.03</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D13" s="3">
+        <v>2684.55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>15</v>
       </c>
@@ -1267,8 +1311,11 @@
       <c r="C14" s="2">
         <v>2.2400000000000002</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D14" s="3">
+        <v>2657.23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>16</v>
       </c>
@@ -1278,8 +1325,11 @@
       <c r="C15" s="2">
         <v>2.88</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D15" s="3">
+        <v>2598.91</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>17</v>
       </c>
@@ -1289,8 +1339,11 @@
       <c r="C16" s="2">
         <v>2.97</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D16" s="3">
+        <v>2526.16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>18</v>
       </c>
@@ -1300,8 +1353,11 @@
       <c r="C17" s="2">
         <v>2.4700000000000002</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D17" s="3">
+        <v>2453.34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>19</v>
       </c>
@@ -1311,8 +1367,11 @@
       <c r="C18" s="2">
         <v>3.23</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D18" s="3">
+        <v>2394.1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>20</v>
       </c>
@@ -1322,8 +1381,11 @@
       <c r="C19" s="2">
         <v>1.64</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D19" s="3">
+        <v>2319.29</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>21</v>
       </c>
@@ -1333,8 +1395,11 @@
       <c r="C20" s="2">
         <v>3.37</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D20" s="3">
+        <v>2281.85</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>22</v>
       </c>
@@ -1344,8 +1409,11 @@
       <c r="C21" s="2">
         <v>3.18</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D21" s="3">
+        <v>2207.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>23</v>
       </c>
@@ -1355,8 +1423,11 @@
       <c r="C22" s="2">
         <v>3.16</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D22" s="3">
+        <v>2139.4699999999998</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>24</v>
       </c>
@@ -1366,8 +1437,11 @@
       <c r="C23" s="2">
         <v>4.53</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D23" s="3">
+        <v>2073.88</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>25</v>
       </c>
@@ -1377,8 +1451,11 @@
       <c r="C24" s="2">
         <v>6.7</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D24" s="3">
+        <v>1984.02</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>26</v>
       </c>
@@ -1388,8 +1465,11 @@
       <c r="C25" s="2">
         <v>2.93</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D25" s="3">
+        <v>1859.38</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>27</v>
       </c>
@@ -1399,8 +1479,11 @@
       <c r="C26" s="2">
         <v>3.28</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D26" s="3">
+        <v>1806.5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>28</v>
       </c>
@@ -1410,8 +1493,11 @@
       <c r="C27" s="2">
         <v>3.43</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D27" s="3">
+        <v>1749.11</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>29</v>
       </c>
@@ -1421,8 +1507,11 @@
       <c r="C28" s="2">
         <v>4.75</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D28" s="3">
+        <v>1691.04</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>30</v>
       </c>
@@ -1432,8 +1521,11 @@
       <c r="C29" s="2">
         <v>9.09</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D29" s="3">
+        <v>1614.31</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>31</v>
       </c>
@@ -1443,8 +1535,11 @@
       <c r="C30" s="2">
         <v>9.49</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D30" s="3">
+        <v>1479.84</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>32</v>
       </c>
@@ -1454,8 +1549,11 @@
       <c r="C31" s="2">
         <v>3.92</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D31" s="3">
+        <v>1351.59</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>33</v>
       </c>
@@ -1465,8 +1563,11 @@
       <c r="C32" s="2">
         <v>0.04</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D32" s="3">
+        <v>1300.5999999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>34</v>
       </c>
@@ -1476,8 +1577,11 @@
       <c r="C33" s="2">
         <v>2.39</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D33" s="3">
+        <v>1300.04</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>35</v>
       </c>
@@ -1487,8 +1591,11 @@
       <c r="C34" s="2">
         <v>2.29</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D34" s="3">
+        <v>1269.75</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>36</v>
       </c>
@@ -1498,8 +1605,11 @@
       <c r="C35" s="2">
         <v>3.15</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D35" s="3">
+        <v>1241.33</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>37</v>
       </c>
@@ -1509,8 +1619,11 @@
       <c r="C36" s="2">
         <v>6.65</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D36" s="3">
+        <v>1203.48</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>38</v>
       </c>
@@ -1520,8 +1633,11 @@
       <c r="C37" s="2">
         <v>1.18</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D37" s="3">
+        <v>1128.45</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>39</v>
       </c>
@@ -1531,8 +1647,11 @@
       <c r="C38" s="2">
         <v>2.88</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D38" s="3">
+        <v>1115.26</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>40</v>
       </c>
@@ -1542,8 +1661,11 @@
       <c r="C39" s="2">
         <v>3.54</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D39" s="3">
+        <v>1084</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>41</v>
       </c>
@@ -1553,8 +1675,11 @@
       <c r="C40" s="2">
         <v>3.08</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D40" s="3">
+        <v>1046.8900000000001</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>42</v>
       </c>
@@ -1564,8 +1689,11 @@
       <c r="C41" s="2">
         <v>1.46</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D41" s="3">
+        <v>1015.65</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>43</v>
       </c>
@@ -1575,8 +1703,11 @@
       <c r="C42" s="2">
         <v>2.37</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D42" s="3">
+        <v>1001.03</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>44</v>
       </c>
@@ -1586,8 +1717,11 @@
       <c r="C43" s="2">
         <v>4.95</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D43" s="3">
+        <v>977.9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>45</v>
       </c>
@@ -1597,8 +1731,11 @@
       <c r="C44" s="2">
         <v>2.98</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D44" s="3">
+        <v>931.76</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>46</v>
       </c>
@@ -1608,8 +1745,11 @@
       <c r="C45" s="2">
         <v>7.25</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D45" s="3">
+        <v>904.79</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>47</v>
       </c>
@@ -1619,8 +1759,11 @@
       <c r="C46" s="2">
         <v>5.46</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D46" s="3">
+        <v>843.64</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>48</v>
       </c>
@@ -1630,8 +1773,11 @@
       <c r="C47" s="2">
         <v>4.8099999999999996</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D47" s="3">
+        <v>799.93</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>49</v>
       </c>
@@ -1641,8 +1787,11 @@
       <c r="C48" s="2">
         <v>11.1</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D48" s="3">
+        <v>763.23</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>50</v>
       </c>
@@ -1652,8 +1801,11 @@
       <c r="C49" s="2">
         <v>13.58</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D49" s="3">
+        <v>686.95</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>51</v>
       </c>
@@ -1663,8 +1815,11 @@
       <c r="C50" s="2">
         <v>3.51</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D50" s="3">
+        <v>604.84</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>52</v>
       </c>
@@ -1674,8 +1829,11 @@
       <c r="C51" s="2">
         <v>2.39</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D51" s="3">
+        <v>584.32000000000005</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>53</v>
       </c>
@@ -1685,8 +1843,11 @@
       <c r="C52" s="2">
         <v>1.25</v>
       </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D52" s="3">
+        <v>570.66</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>54</v>
       </c>
@@ -1696,8 +1857,11 @@
       <c r="C53" s="2">
         <v>1.1200000000000001</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D53" s="3">
+        <v>563.6</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>55</v>
       </c>
@@ -1707,8 +1871,11 @@
       <c r="C54" s="2">
         <v>1.8</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D54" s="3">
+        <v>557.36</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>56</v>
       </c>
@@ -1718,8 +1885,11 @@
       <c r="C55" s="2">
         <v>1.94</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D55" s="3">
+        <v>547.48</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>57</v>
       </c>
@@ -1729,8 +1899,11 @@
       <c r="C56" s="2">
         <v>0.89</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D56" s="3">
+        <v>537.04999999999995</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>58</v>
       </c>
@@ -1740,8 +1913,11 @@
       <c r="C57" s="2">
         <v>1.68</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D57" s="3">
+        <v>532.32000000000005</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>59</v>
       </c>
@@ -1751,8 +1927,11 @@
       <c r="C58" s="2">
         <v>1.08</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D58" s="3">
+        <v>523.53</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>60</v>
       </c>
@@ -1762,8 +1941,11 @@
       <c r="C59" s="2">
         <v>0.91</v>
       </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D59" s="3">
+        <v>517.96</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>61</v>
       </c>
@@ -1773,8 +1955,11 @@
       <c r="C60" s="2">
         <v>1.68</v>
       </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D60" s="3">
+        <v>513.29999999999995</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>62</v>
       </c>
@@ -1784,8 +1969,11 @@
       <c r="C61" s="2">
         <v>1.25</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D61" s="3">
+        <v>504.81</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>63</v>
       </c>
@@ -1795,8 +1983,11 @@
       <c r="C62" s="2">
         <v>2.2999999999999998</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D62" s="3">
+        <v>498.58</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>64</v>
       </c>
@@ -1806,8 +1997,11 @@
       <c r="C63" s="2">
         <v>2.13</v>
       </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D63" s="3">
+        <v>487.38</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>65</v>
       </c>
@@ -1817,8 +2011,11 @@
       <c r="C64" s="2">
         <v>0.97</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D64" s="3">
+        <v>477.21</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>66</v>
       </c>
@@ -1828,8 +2025,11 @@
       <c r="C65" s="2">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D65" s="3">
+        <v>472.61</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>67</v>
       </c>
@@ -1839,8 +2039,11 @@
       <c r="C66" s="2">
         <v>0.57999999999999996</v>
       </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D66" s="3">
+        <v>468.56</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>68</v>
       </c>
@@ -1850,8 +2053,11 @@
       <c r="C67" s="2">
         <v>1.1299999999999999</v>
       </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D67" s="3">
+        <v>465.84</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>69</v>
       </c>
@@ -1861,8 +2067,11 @@
       <c r="C68" s="2">
         <v>1.36</v>
       </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D68" s="3">
+        <v>460.62</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>70</v>
       </c>
@@ -1872,8 +2081,11 @@
       <c r="C69" s="2">
         <v>0.85</v>
       </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D69" s="3">
+        <v>454.43</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>71</v>
       </c>
@@ -1883,8 +2095,11 @@
       <c r="C70" s="2">
         <v>0.56999999999999995</v>
       </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D70" s="3">
+        <v>450.58</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>72</v>
       </c>
@@ -1894,8 +2109,11 @@
       <c r="C71" s="2">
         <v>0.35</v>
       </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D71" s="3">
+        <v>448.02</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>73</v>
       </c>
@@ -1905,8 +2123,11 @@
       <c r="C72" s="2">
         <v>1.35</v>
       </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D72" s="3">
+        <v>446.45</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>74</v>
       </c>
@@ -1916,8 +2137,11 @@
       <c r="C73" s="2">
         <v>0.74</v>
       </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D73" s="3">
+        <v>440.5</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>75</v>
       </c>
@@ -1927,8 +2151,11 @@
       <c r="C74" s="2">
         <v>0.38</v>
       </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D74" s="3">
+        <v>437.25</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>76</v>
       </c>
@@ -1938,8 +2165,11 @@
       <c r="C75" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D75" s="3">
+        <v>435.59</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>77</v>
       </c>
@@ -1949,8 +2179,11 @@
       <c r="C76" s="2">
         <v>0.99</v>
       </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D76" s="3">
+        <v>427.04</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>78</v>
       </c>
@@ -1960,8 +2193,11 @@
       <c r="C77" s="2">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D77" s="3">
+        <v>422.84</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>79</v>
       </c>
@@ -1971,8 +2207,11 @@
       <c r="C78" s="2">
         <v>1.36</v>
       </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D78" s="3">
+        <v>419.24</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>80</v>
       </c>
@@ -1982,8 +2221,11 @@
       <c r="C79" s="2">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D79" s="3">
+        <v>413.63</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>81</v>
       </c>
@@ -1993,8 +2235,11 @@
       <c r="C80" s="2">
         <v>0.95</v>
       </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D80" s="3">
+        <v>413.52</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>82</v>
       </c>
@@ -2004,8 +2249,11 @@
       <c r="C81" s="2">
         <v>1.69</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D81" s="3">
+        <v>409.63</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>83</v>
       </c>
@@ -2015,8 +2263,11 @@
       <c r="C82" s="2">
         <v>1.03</v>
       </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D82" s="3">
+        <v>402.81</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>84</v>
       </c>
@@ -2026,8 +2277,11 @@
       <c r="C83" s="2">
         <v>0.16</v>
       </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D83" s="3">
+        <v>398.71</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>85</v>
       </c>
@@ -2037,8 +2291,11 @@
       <c r="C84" s="2">
         <v>1.06</v>
       </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D84" s="3">
+        <v>398.07</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>86</v>
       </c>
@@ -2048,8 +2305,11 @@
       <c r="C85" s="2">
         <v>-0.4</v>
       </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D85" s="3">
+        <v>393.88</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>87</v>
       </c>
@@ -2059,8 +2319,11 @@
       <c r="C86" s="2">
         <v>-1.44</v>
       </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D86" s="3">
+        <v>395.48</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>88</v>
       </c>
@@ -2070,8 +2333,11 @@
       <c r="C87" s="2">
         <v>2.67</v>
       </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D87" s="3">
+        <v>401.27</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>89</v>
       </c>
@@ -2081,8 +2347,11 @@
       <c r="C88" s="2">
         <v>6.3</v>
       </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D88" s="3">
+        <v>390.84</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>90</v>
       </c>
@@ -2092,8 +2361,11 @@
       <c r="C89" s="2">
         <v>2.2999999999999998</v>
       </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D89" s="3">
+        <v>367.66</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>91</v>
       </c>
@@ -2103,8 +2375,11 @@
       <c r="C90" s="2">
         <v>0.55000000000000004</v>
       </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D90" s="3">
+        <v>359.41</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>92</v>
       </c>
@@ -2114,8 +2389,11 @@
       <c r="C91" s="2">
         <v>2.61</v>
       </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D91" s="3">
+        <v>357.44</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>93</v>
       </c>
@@ -2125,8 +2403,11 @@
       <c r="C92" s="2">
         <v>1.62</v>
       </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D92" s="3">
+        <v>348.34</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>94</v>
       </c>
@@ -2136,8 +2417,11 @@
       <c r="C93" s="2">
         <v>1.87</v>
       </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D93" s="3">
+        <v>342.78</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>95</v>
       </c>
@@ -2147,8 +2431,11 @@
       <c r="C94" s="2">
         <v>0.99</v>
       </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D94" s="3">
+        <v>336.48</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>96</v>
       </c>
@@ -2158,8 +2445,11 @@
       <c r="C95" s="2">
         <v>0.73</v>
       </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D95" s="3">
+        <v>333.17</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>97</v>
       </c>
@@ -2169,8 +2459,11 @@
       <c r="C96" s="2">
         <v>1.02</v>
       </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D96" s="3">
+        <v>330.75</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>98</v>
       </c>
@@ -2180,8 +2473,11 @@
       <c r="C97" s="2">
         <v>0.69</v>
       </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D97" s="3">
+        <v>327.41000000000003</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>99</v>
       </c>
@@ -2191,8 +2487,11 @@
       <c r="C98" s="2">
         <v>1.49</v>
       </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D98" s="3">
+        <v>325.18</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>100</v>
       </c>
@@ -2202,8 +2501,11 @@
       <c r="C99" s="2">
         <v>2.08</v>
       </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D99" s="3">
+        <v>320.39999999999998</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>101</v>
       </c>
@@ -2213,8 +2515,11 @@
       <c r="C100" s="2">
         <v>0.65</v>
       </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D100" s="3">
+        <v>313.88</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>102</v>
       </c>
@@ -2224,8 +2529,11 @@
       <c r="C101" s="2">
         <v>0.52</v>
       </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D101" s="3">
+        <v>311.85000000000002</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>103</v>
       </c>
@@ -2235,8 +2543,11 @@
       <c r="C102" s="2">
         <v>0.15</v>
       </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D102" s="3">
+        <v>310.24</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>104</v>
       </c>
@@ -2246,8 +2557,11 @@
       <c r="C103" s="2">
         <v>-0.27</v>
       </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D103" s="3">
+        <v>309.77999999999997</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>105</v>
       </c>
@@ -2257,8 +2571,11 @@
       <c r="C104" s="2">
         <v>0.45</v>
       </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D104" s="3">
+        <v>310.61</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>106</v>
       </c>
@@ -2268,8 +2585,11 @@
       <c r="C105" s="2">
         <v>1.31</v>
       </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D105" s="3">
+        <v>309.23</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>107</v>
       </c>
@@ -2279,8 +2599,11 @@
       <c r="C106" s="2">
         <v>1.02</v>
       </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D106" s="3">
+        <v>305.24</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>108</v>
       </c>
@@ -2290,8 +2613,11 @@
       <c r="C107" s="2">
         <v>0.81</v>
       </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D107" s="3">
+        <v>302.17</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>109</v>
       </c>
@@ -2301,8 +2627,11 @@
       <c r="C108" s="2">
         <v>2.46</v>
       </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D108" s="3">
+        <v>299.74</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>110</v>
       </c>
@@ -2312,8 +2641,11 @@
       <c r="C109" s="2">
         <v>1.64</v>
       </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D109" s="3">
+        <v>292.54000000000002</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>111</v>
       </c>
@@ -2323,8 +2655,11 @@
       <c r="C110" s="2">
         <v>0.52</v>
       </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D110" s="3">
+        <v>287.81</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>112</v>
       </c>
@@ -2334,8 +2669,11 @@
       <c r="C111" s="2">
         <v>1.44</v>
       </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D111" s="3">
+        <v>286.33</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>113</v>
       </c>
@@ -2345,8 +2683,11 @@
       <c r="C112" s="2">
         <v>0.18</v>
       </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D112" s="3">
+        <v>282.27</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>114</v>
       </c>
@@ -2356,8 +2697,11 @@
       <c r="C113" s="2">
         <v>-0.28999999999999998</v>
       </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D113" s="3">
+        <v>281.76</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>115</v>
       </c>
@@ -2367,8 +2711,11 @@
       <c r="C114" s="2">
         <v>1.1599999999999999</v>
       </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D114" s="3">
+        <v>282.58</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
         <v>116</v>
       </c>
@@ -2378,8 +2725,11 @@
       <c r="C115" s="2">
         <v>0.47</v>
       </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D115" s="3">
+        <v>279.33</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
         <v>117</v>
       </c>
@@ -2389,8 +2739,11 @@
       <c r="C116" s="2">
         <v>0.57999999999999996</v>
       </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D116" s="3">
+        <v>278.02</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>118</v>
       </c>
@@ -2400,8 +2753,11 @@
       <c r="C117" s="2">
         <v>0.78</v>
       </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D117" s="3">
+        <v>276.42</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
         <v>119</v>
       </c>
@@ -2411,8 +2767,11 @@
       <c r="C118" s="2">
         <v>-0.04</v>
       </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D118" s="3">
+        <v>274.27</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
         <v>120</v>
       </c>
@@ -2422,8 +2781,11 @@
       <c r="C119" s="2">
         <v>-0.02</v>
       </c>
-    </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D119" s="3">
+        <v>274.38</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
         <v>121</v>
       </c>
@@ -2433,8 +2795,11 @@
       <c r="C120" s="2">
         <v>1.82</v>
       </c>
-    </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D120" s="3">
+        <v>274.44</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
         <v>122</v>
       </c>
@@ -2444,8 +2809,11 @@
       <c r="C121" s="2">
         <v>0.21</v>
       </c>
-    </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D121" s="3">
+        <v>269.54000000000002</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
         <v>123</v>
       </c>
@@ -2455,8 +2823,11 @@
       <c r="C122" s="2">
         <v>0.67</v>
       </c>
-    </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D122" s="3">
+        <v>268.98</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>124</v>
       </c>
@@ -2466,8 +2837,11 @@
       <c r="C123" s="2">
         <v>1.55</v>
       </c>
-    </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D123" s="3">
+        <v>267.2</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
         <v>125</v>
       </c>
@@ -2477,8 +2851,11 @@
       <c r="C124" s="2">
         <v>0.89</v>
       </c>
-    </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D124" s="3">
+        <v>263.11</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
         <v>126</v>
       </c>
@@ -2488,8 +2865,11 @@
       <c r="C125" s="2">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D125" s="3">
+        <v>260.77999999999997</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
         <v>127</v>
       </c>
@@ -2499,8 +2879,11 @@
       <c r="C126" s="2">
         <v>0.09</v>
       </c>
-    </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D126" s="3">
+        <v>259.74</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>128</v>
       </c>
@@ -2510,8 +2893,11 @@
       <c r="C127" s="2">
         <v>-0.51</v>
       </c>
-    </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D127" s="3">
+        <v>259.51</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A128" s="1" t="s">
         <v>129</v>
       </c>
@@ -2521,8 +2907,11 @@
       <c r="C128" s="2">
         <v>0.56000000000000005</v>
       </c>
-    </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D128" s="3">
+        <v>260.85000000000002</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
         <v>130</v>
       </c>
@@ -2532,8 +2921,11 @@
       <c r="C129" s="2">
         <v>1.63</v>
       </c>
-    </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D129" s="3">
+        <v>259.39</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
         <v>131</v>
       </c>
@@ -2543,8 +2935,11 @@
       <c r="C130" s="2">
         <v>1.19</v>
       </c>
-    </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D130" s="3">
+        <v>255.23</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
         <v>132</v>
       </c>
@@ -2554,8 +2949,11 @@
       <c r="C131" s="2">
         <v>0.71</v>
       </c>
-    </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D131" s="3">
+        <v>252.24</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>133</v>
       </c>
@@ -2565,8 +2963,11 @@
       <c r="C132" s="2">
         <v>1.1000000000000001</v>
       </c>
-    </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D132" s="3">
+        <v>250.45</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
         <v>134</v>
       </c>
@@ -2576,8 +2977,11 @@
       <c r="C133" s="2">
         <v>-0.44</v>
       </c>
-    </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D133" s="3">
+        <v>247.72</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
         <v>135</v>
       </c>
@@ -2587,8 +2991,11 @@
       <c r="C134" s="2">
         <v>0.18</v>
       </c>
-    </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D134" s="3">
+        <v>248.82</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>136</v>
       </c>
@@ -2598,8 +3005,11 @@
       <c r="C135" s="2">
         <v>1.9</v>
       </c>
-    </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D135" s="3">
+        <v>248.37</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>137</v>
       </c>
@@ -2609,8 +3019,11 @@
       <c r="C136" s="2">
         <v>0.14000000000000001</v>
       </c>
-    </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D136" s="3">
+        <v>243.74</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>138</v>
       </c>
@@ -2620,8 +3033,11 @@
       <c r="C137" s="2">
         <v>0.09</v>
       </c>
-    </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D137" s="3">
+        <v>243.4</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>139</v>
       </c>
@@ -2631,8 +3047,11 @@
       <c r="C138" s="2">
         <v>0.45</v>
       </c>
-    </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D138" s="3">
+        <v>243.17</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
         <v>140</v>
       </c>
@@ -2642,8 +3061,11 @@
       <c r="C139" s="2">
         <v>0.31</v>
       </c>
-    </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D139" s="3">
+        <v>242.07</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
         <v>141</v>
       </c>
@@ -2653,8 +3075,11 @@
       <c r="C140" s="2">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D140" s="3">
+        <v>241.32</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
         <v>142</v>
       </c>
@@ -2664,8 +3089,11 @@
       <c r="C141" s="2">
         <v>1.34</v>
       </c>
-    </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D141" s="3">
+        <v>240.37</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A142" s="1" t="s">
         <v>143</v>
       </c>
@@ -2675,8 +3103,11 @@
       <c r="C142" s="2">
         <v>1.1299999999999999</v>
       </c>
-    </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D142" s="3">
+        <v>237.18</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
         <v>144</v>
       </c>
@@ -2686,8 +3117,11 @@
       <c r="C143" s="2">
         <v>0.43</v>
       </c>
-    </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D143" s="3">
+        <v>234.54</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
         <v>145</v>
       </c>
@@ -2697,8 +3131,11 @@
       <c r="C144" s="2">
         <v>1.98</v>
       </c>
-    </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D144" s="3">
+        <v>233.54</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>146</v>
       </c>
@@ -2708,8 +3145,11 @@
       <c r="C145" s="2">
         <v>0.46</v>
       </c>
-    </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D145" s="3">
+        <v>229.01</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>147</v>
       </c>
@@ -2719,8 +3159,11 @@
       <c r="C146" s="2">
         <v>0.01</v>
       </c>
-    </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D146" s="3">
+        <v>227.96</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
         <v>148</v>
       </c>
@@ -2730,8 +3173,11 @@
       <c r="C147" s="2">
         <v>1.8</v>
       </c>
-    </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D147" s="3">
+        <v>227.94</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
         <v>149</v>
       </c>
@@ -2741,8 +3187,11 @@
       <c r="C148" s="2">
         <v>0.77</v>
       </c>
-    </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D148" s="3">
+        <v>223.91</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>150</v>
       </c>
@@ -2752,8 +3201,11 @@
       <c r="C149" s="2">
         <v>-0.1</v>
       </c>
-    </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D149" s="3">
+        <v>222.21</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
         <v>151</v>
       </c>
@@ -2763,8 +3215,11 @@
       <c r="C150" s="2">
         <v>0.31</v>
       </c>
-    </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D150" s="3">
+        <v>222.44</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
         <v>152</v>
       </c>
@@ -2774,8 +3229,11 @@
       <c r="C151" s="2">
         <v>0.76</v>
       </c>
-    </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D151" s="3">
+        <v>221.75</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A152" s="1" t="s">
         <v>153</v>
       </c>
@@ -2785,8 +3243,11 @@
       <c r="C152" s="2">
         <v>0.15</v>
       </c>
-    </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D152" s="3">
+        <v>220.07</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
         <v>154</v>
       </c>
@@ -2796,8 +3257,11 @@
       <c r="C153" s="2">
         <v>0.42</v>
       </c>
-    </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D153" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A154" s="1" t="s">
         <v>155</v>
       </c>
@@ -2807,8 +3271,11 @@
       <c r="C154" s="2">
         <v>0.66</v>
       </c>
-    </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D154" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
         <v>156</v>
       </c>
@@ -2818,8 +3285,11 @@
       <c r="C155" s="2">
         <v>0.3</v>
       </c>
-    </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D155" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
         <v>157</v>
       </c>
@@ -2829,8 +3299,11 @@
       <c r="C156" s="2">
         <v>1.65</v>
       </c>
-    </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D156" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
         <v>158</v>
       </c>
@@ -2840,8 +3313,11 @@
       <c r="C157" s="2">
         <v>0.38</v>
       </c>
-    </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D157" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
         <v>159</v>
       </c>
@@ -2851,8 +3327,11 @@
       <c r="C158" s="2">
         <v>0.38</v>
       </c>
-    </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D158" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
         <v>160</v>
       </c>
@@ -2862,8 +3341,11 @@
       <c r="C159" s="2">
         <v>1.96</v>
       </c>
-    </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D159" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
         <v>161</v>
       </c>
@@ -2873,8 +3355,11 @@
       <c r="C160" s="2">
         <v>1.03</v>
       </c>
-    </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D160" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
         <v>162</v>
       </c>
@@ -2884,8 +3369,11 @@
       <c r="C161" s="2">
         <v>0.56000000000000005</v>
       </c>
-    </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D161" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A162" s="1" t="s">
         <v>163</v>
       </c>
@@ -2895,8 +3383,11 @@
       <c r="C162" s="2">
         <v>-0.23</v>
       </c>
-    </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D162" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A163" s="1" t="s">
         <v>164</v>
       </c>
@@ -2906,8 +3397,11 @@
       <c r="C163" s="2">
         <v>-0.9</v>
       </c>
-    </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D163" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
         <v>165</v>
       </c>
@@ -2917,8 +3411,11 @@
       <c r="C164" s="2">
         <v>-0.21</v>
       </c>
-    </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D164" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
         <v>166</v>
       </c>
@@ -2928,8 +3425,11 @@
       <c r="C165" s="2">
         <v>1.52</v>
       </c>
-    </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D165" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
         <v>167</v>
       </c>
@@ -2939,8 +3439,11 @@
       <c r="C166" s="2">
         <v>0.41</v>
       </c>
-    </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D166" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
         <v>168</v>
       </c>
@@ -2950,8 +3453,11 @@
       <c r="C167" s="2">
         <v>0.56000000000000005</v>
       </c>
-    </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D167" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A168" s="1" t="s">
         <v>169</v>
       </c>
@@ -2961,8 +3467,11 @@
       <c r="C168" s="2">
         <v>0.56000000000000005</v>
       </c>
-    </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D168" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A169" s="1" t="s">
         <v>170</v>
       </c>
@@ -2972,8 +3481,11 @@
       <c r="C169" s="2">
         <v>0.57999999999999996</v>
       </c>
-    </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D169" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A170" s="1" t="s">
         <v>171</v>
       </c>
@@ -2983,8 +3495,11 @@
       <c r="C170" s="2">
         <v>1.73</v>
       </c>
-    </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D170" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A171" s="1" t="s">
         <v>172</v>
       </c>
@@ -2994,8 +3509,11 @@
       <c r="C171" s="2">
         <v>3.27</v>
       </c>
-    </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D171" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A172" s="1" t="s">
         <v>173</v>
       </c>
@@ -3005,8 +3523,11 @@
       <c r="C172" s="2">
         <v>0.75</v>
       </c>
-    </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D172" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A173" s="1" t="s">
         <v>174</v>
       </c>
@@ -3016,8 +3537,11 @@
       <c r="C173" s="2">
         <v>0.73</v>
       </c>
-    </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D173" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A174" s="1" t="s">
         <v>175</v>
       </c>
@@ -3027,8 +3551,11 @@
       <c r="C174" s="2">
         <v>-0.41</v>
       </c>
-    </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D174" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A175" s="1" t="s">
         <v>176</v>
       </c>
@@ -3038,8 +3565,11 @@
       <c r="C175" s="2">
         <v>-1.43</v>
       </c>
-    </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D175" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A176" s="1" t="s">
         <v>177</v>
       </c>
@@ -3049,8 +3579,11 @@
       <c r="C176" s="2">
         <v>2.42</v>
       </c>
-    </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D176" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A177" s="1" t="s">
         <v>178</v>
       </c>
@@ -3060,8 +3593,11 @@
       <c r="C177" s="2">
         <v>0.87</v>
       </c>
-    </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D177" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A178" s="1" t="s">
         <v>179</v>
       </c>
@@ -3071,8 +3607,11 @@
       <c r="C178" s="2">
         <v>0.42</v>
       </c>
-    </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D178" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A179" s="1" t="s">
         <v>180</v>
       </c>
@@ -3082,8 +3621,11 @@
       <c r="C179" s="2">
         <v>0.73</v>
       </c>
-    </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D179" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A180" s="1" t="s">
         <v>181</v>
       </c>
@@ -3093,8 +3635,11 @@
       <c r="C180" s="2">
         <v>0.41</v>
       </c>
-    </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D180" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A181" s="1" t="s">
         <v>182</v>
       </c>
@@ -3104,8 +3649,11 @@
       <c r="C181" s="2">
         <v>-0.3</v>
       </c>
-    </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D181" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A182" s="1" t="s">
         <v>183</v>
       </c>
@@ -3115,8 +3663,11 @@
       <c r="C182" s="2">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D182" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A183" s="1" t="s">
         <v>184</v>
       </c>
@@ -3126,8 +3677,11 @@
       <c r="C183" s="2">
         <v>1.83</v>
       </c>
-    </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D183" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A184" s="1" t="s">
         <v>185</v>
       </c>
@@ -3137,8 +3691,11 @@
       <c r="C184" s="2">
         <v>1.23</v>
       </c>
-    </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D184" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A185" s="1" t="s">
         <v>186</v>
       </c>
@@ -3148,8 +3705,11 @@
       <c r="C185" s="2">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D185" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A186" s="1" t="s">
         <v>187</v>
       </c>
@@ -3159,8 +3719,11 @@
       <c r="C186" s="2">
         <v>-0.48</v>
       </c>
-    </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D186" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A187" s="1" t="s">
         <v>188</v>
       </c>
@@ -3170,8 +3733,11 @@
       <c r="C187" s="2">
         <v>-0.56000000000000005</v>
       </c>
-    </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D187" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A188" s="1" t="s">
         <v>189</v>
       </c>
@@ -3181,8 +3747,11 @@
       <c r="C188" s="2">
         <v>-0.36</v>
       </c>
-    </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D188" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A189" s="1" t="s">
         <v>190</v>
       </c>
@@ -3192,8 +3761,11 @@
       <c r="C189" s="2">
         <v>0.6</v>
       </c>
-    </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D189" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A190" s="1" t="s">
         <v>191</v>
       </c>
@@ -3203,8 +3775,11 @@
       <c r="C190" s="2">
         <v>0.57999999999999996</v>
       </c>
-    </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D190" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A191" s="1" t="s">
         <v>192</v>
       </c>
@@ -3214,8 +3789,11 @@
       <c r="C191" s="2">
         <v>1.45</v>
       </c>
-    </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D191" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A192" s="1" t="s">
         <v>193</v>
       </c>
@@ -3225,8 +3803,11 @@
       <c r="C192" s="2">
         <v>1.85</v>
       </c>
-    </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D192" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A193" s="1" t="s">
         <v>194</v>
       </c>
@@ -3236,8 +3817,11 @@
       <c r="C193" s="2">
         <v>0.53</v>
       </c>
-    </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D193" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A194" s="1" t="s">
         <v>195</v>
       </c>
@@ -3247,8 +3831,11 @@
       <c r="C194" s="2">
         <v>1.27</v>
       </c>
-    </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D194" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A195" s="1" t="s">
         <v>196</v>
       </c>
@@ -3258,8 +3845,11 @@
       <c r="C195" s="2">
         <v>2.41</v>
       </c>
-    </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D195" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="196" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A196" s="1" t="s">
         <v>197</v>
       </c>
@@ -3269,8 +3859,11 @@
       <c r="C196" s="2">
         <v>0.39</v>
       </c>
-    </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D196" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A197" s="1" t="s">
         <v>198</v>
       </c>
@@ -3280,8 +3873,11 @@
       <c r="C197" s="2">
         <v>-0.3</v>
       </c>
-    </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D197" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A198" s="1" t="s">
         <v>199</v>
       </c>
@@ -3291,8 +3887,11 @@
       <c r="C198" s="2">
         <v>0.25</v>
       </c>
-    </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D198" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="199" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A199" s="1" t="s">
         <v>200</v>
       </c>
@@ -3302,8 +3901,11 @@
       <c r="C199" s="2">
         <v>0.11</v>
       </c>
-    </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D199" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A200" s="1" t="s">
         <v>201</v>
       </c>
@@ -3313,8 +3915,11 @@
       <c r="C200" s="2">
         <v>0.64</v>
       </c>
-    </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D200" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A201" s="1" t="s">
         <v>202</v>
       </c>
@@ -3324,8 +3929,11 @@
       <c r="C201" s="2">
         <v>0.02</v>
       </c>
-    </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D201" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A202" s="1" t="s">
         <v>203</v>
       </c>
@@ -3335,8 +3943,11 @@
       <c r="C202" s="2">
         <v>1.1000000000000001</v>
       </c>
-    </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D202" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="203" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A203" s="1" t="s">
         <v>204</v>
       </c>
@@ -3346,8 +3957,11 @@
       <c r="C203" s="2">
         <v>-0.34</v>
       </c>
-    </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D203" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="204" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A204" s="1" t="s">
         <v>205</v>
       </c>
@@ -3357,8 +3971,11 @@
       <c r="C204" s="2">
         <v>0.28999999999999998</v>
       </c>
-    </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D204" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="205" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A205" s="1" t="s">
         <v>206</v>
       </c>
@@ -3368,8 +3985,11 @@
       <c r="C205" s="2">
         <v>-0.41</v>
       </c>
-    </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D205" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="206" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A206" s="1" t="s">
         <v>207</v>
       </c>
@@ -3379,8 +3999,11 @@
       <c r="C206" s="2">
         <v>0.83</v>
       </c>
-    </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D206" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="207" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A207" s="1" t="s">
         <v>208</v>
       </c>
@@ -3390,8 +4013,11 @@
       <c r="C207" s="2">
         <v>2.6</v>
       </c>
-    </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D207" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="208" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A208" s="1" t="s">
         <v>209</v>
       </c>
@@ -3401,8 +4027,11 @@
       <c r="C208" s="2">
         <v>0.45</v>
       </c>
-    </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D208" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A209" s="1" t="s">
         <v>210</v>
       </c>
@@ -3412,8 +4041,11 @@
       <c r="C209" s="2">
         <v>-0.24</v>
       </c>
-    </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D209" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="210" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A210" s="1" t="s">
         <v>211</v>
       </c>
@@ -3423,8 +4055,11 @@
       <c r="C210" s="2">
         <v>0.57999999999999996</v>
       </c>
-    </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D210" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="211" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A211" s="1" t="s">
         <v>212</v>
       </c>
@@ -3434,8 +4069,11 @@
       <c r="C211" s="2">
         <v>-0.36</v>
       </c>
-    </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D211" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="212" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A212" s="1" t="s">
         <v>213</v>
       </c>
@@ -3445,8 +4083,11 @@
       <c r="C212" s="2">
         <v>1.49</v>
       </c>
-    </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D212" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A213" s="1" t="s">
         <v>214</v>
       </c>
@@ -3456,8 +4097,11 @@
       <c r="C213" s="2">
         <v>1.68</v>
       </c>
-    </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D213" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A214" s="1" t="s">
         <v>215</v>
       </c>
@@ -3467,8 +4111,11 @@
       <c r="C214" s="2">
         <v>0.96</v>
       </c>
-    </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D214" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="215" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A215" s="1" t="s">
         <v>216</v>
       </c>
@@ -3478,8 +4125,11 @@
       <c r="C215" s="2">
         <v>1.29</v>
       </c>
-    </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D215" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="216" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A216" s="1" t="s">
         <v>217</v>
       </c>
@@ -3489,8 +4139,11 @@
       <c r="C216" s="2">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D216" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="217" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A217" s="1" t="s">
         <v>218</v>
       </c>
@@ -3500,8 +4153,11 @@
       <c r="C217" s="2">
         <v>0.22</v>
       </c>
-    </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D217" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A218" s="1" t="s">
         <v>219</v>
       </c>
@@ -3511,8 +4167,11 @@
       <c r="C218" s="2">
         <v>1.95</v>
       </c>
-    </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D218" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="219" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A219" s="1" t="s">
         <v>220</v>
       </c>
@@ -3522,8 +4181,11 @@
       <c r="C219" s="2">
         <v>1.81</v>
       </c>
-    </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D219" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="220" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A220" s="1" t="s">
         <v>221</v>
       </c>
@@ -3533,8 +4195,11 @@
       <c r="C220" s="2">
         <v>1.03</v>
       </c>
-    </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D220" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="221" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A221" s="1" t="s">
         <v>222</v>
       </c>
@@ -3544,8 +4209,11 @@
       <c r="C221" s="2">
         <v>0.02</v>
       </c>
-    </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D221" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A222" s="1" t="s">
         <v>223</v>
       </c>
@@ -3555,8 +4223,11 @@
       <c r="C222" s="2">
         <v>-0.73</v>
       </c>
-    </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D222" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A223" s="1" t="s">
         <v>224</v>
       </c>
@@ -3566,8 +4237,11 @@
       <c r="C223" s="2">
         <v>-0.24</v>
       </c>
-    </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D223" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="224" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A224" s="1" t="s">
         <v>225</v>
       </c>
@@ -3577,8 +4251,11 @@
       <c r="C224" s="2">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D224" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A225" s="1" t="s">
         <v>226</v>
       </c>
@@ -3588,8 +4265,11 @@
       <c r="C225" s="2">
         <v>1.21</v>
       </c>
-    </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D225" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="226" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A226" s="1" t="s">
         <v>227</v>
       </c>
@@ -3599,8 +4279,11 @@
       <c r="C226" s="2">
         <v>0.92</v>
       </c>
-    </row>
-    <row r="227" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D226" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A227" s="1" t="s">
         <v>228</v>
       </c>
@@ -3610,8 +4293,11 @@
       <c r="C227" s="2">
         <v>0.43</v>
       </c>
-    </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D227" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A228" s="1" t="s">
         <v>229</v>
       </c>
@@ -3621,8 +4307,11 @@
       <c r="C228" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D228" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="229" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A229" s="1" t="s">
         <v>230</v>
       </c>
@@ -3632,8 +4321,11 @@
       <c r="C229" s="2">
         <v>0.23</v>
       </c>
-    </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D229" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="230" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A230" s="1" t="s">
         <v>231</v>
       </c>
@@ -3643,8 +4335,11 @@
       <c r="C230" s="2">
         <v>1.29</v>
       </c>
-    </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D230" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="231" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A231" s="1" t="s">
         <v>232</v>
       </c>
@@ -3654,8 +4349,11 @@
       <c r="C231" s="2">
         <v>1.27</v>
       </c>
-    </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D231" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="232" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A232" s="1" t="s">
         <v>233</v>
       </c>
@@ -3665,8 +4363,11 @@
       <c r="C232" s="2">
         <v>1.29</v>
       </c>
-    </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D232" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="233" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A233" s="1" t="s">
         <v>234</v>
       </c>
@@ -3676,8 +4377,11 @@
       <c r="C233" s="2">
         <v>-0.44</v>
       </c>
-    </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D233" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="234" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A234" s="1" t="s">
         <v>235</v>
       </c>
@@ -3687,8 +4391,11 @@
       <c r="C234" s="2">
         <v>0.85</v>
       </c>
-    </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D234" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="235" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A235" s="1" t="s">
         <v>236</v>
       </c>
@@ -3698,8 +4405,11 @@
       <c r="C235" s="2">
         <v>0.34</v>
       </c>
-    </row>
-    <row r="236" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D235" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="236" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A236" s="1" t="s">
         <v>237</v>
       </c>
@@ -3709,8 +4419,11 @@
       <c r="C236" s="2">
         <v>1.88</v>
       </c>
-    </row>
-    <row r="237" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D236" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="237" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A237" s="1" t="s">
         <v>238</v>
       </c>
@@ -3720,8 +4433,11 @@
       <c r="C237" s="2">
         <v>1.34</v>
       </c>
-    </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D237" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="238" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A238" s="1" t="s">
         <v>239</v>
       </c>
@@ -3731,8 +4447,11 @@
       <c r="C238" s="2">
         <v>0.27</v>
       </c>
-    </row>
-    <row r="239" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D238" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="239" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A239" s="1" t="s">
         <v>240</v>
       </c>
@@ -3742,8 +4461,11 @@
       <c r="C239" s="2">
         <v>0.22</v>
       </c>
-    </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D239" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="240" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A240" s="1" t="s">
         <v>241</v>
       </c>
@@ -3753,8 +4475,11 @@
       <c r="C240" s="2">
         <v>0.75</v>
       </c>
-    </row>
-    <row r="241" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D240" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="241" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A241" s="1" t="s">
         <v>242</v>
       </c>
@@ -3764,8 +4489,11 @@
       <c r="C241" s="2">
         <v>0.42</v>
       </c>
-    </row>
-    <row r="242" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D241" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="242" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A242" s="1" t="s">
         <v>243</v>
       </c>
@@ -3775,8 +4503,11 @@
       <c r="C242" s="2">
         <v>1.4</v>
       </c>
-    </row>
-    <row r="243" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D242" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="243" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A243" s="1" t="s">
         <v>244</v>
       </c>
@@ -3786,8 +4517,11 @@
       <c r="C243" s="2">
         <v>1.79</v>
       </c>
-    </row>
-    <row r="244" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D243" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="244" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A244" s="1" t="s">
         <v>245</v>
       </c>
@@ -3797,8 +4531,11 @@
       <c r="C244" s="2">
         <v>1.02</v>
       </c>
-    </row>
-    <row r="245" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D244" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="245" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A245" s="1" t="s">
         <v>246</v>
       </c>
@@ -3808,8 +4545,11 @@
       <c r="C245" s="2">
         <v>0.85</v>
       </c>
-    </row>
-    <row r="246" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D245" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="246" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A246" s="1" t="s">
         <v>247</v>
       </c>
@@ -3819,8 +4559,11 @@
       <c r="C246" s="2">
         <v>-0.56999999999999995</v>
       </c>
-    </row>
-    <row r="247" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D246" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="247" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A247" s="1" t="s">
         <v>248</v>
       </c>
@@ -3830,8 +4573,11 @@
       <c r="C247" s="2">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="248" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D247" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="248" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A248" s="1" t="s">
         <v>249</v>
       </c>
@@ -3841,8 +4587,11 @@
       <c r="C248" s="2">
         <v>0.92</v>
       </c>
-    </row>
-    <row r="249" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D248" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="249" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A249" s="1" t="s">
         <v>250</v>
       </c>
@@ -3852,8 +4601,11 @@
       <c r="C249" s="2">
         <v>0.71</v>
       </c>
-    </row>
-    <row r="250" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D249" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="250" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A250" s="1" t="s">
         <v>251</v>
       </c>
@@ -3863,8 +4615,11 @@
       <c r="C250" s="2">
         <v>0.26</v>
       </c>
-    </row>
-    <row r="251" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D250" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="251" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A251" s="1" t="s">
         <v>252</v>
       </c>
@@ -3874,8 +4629,11 @@
       <c r="C251" s="2">
         <v>0.02</v>
       </c>
-    </row>
-    <row r="252" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D251" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="252" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A252" s="1" t="s">
         <v>253</v>
       </c>
@@ -3884,6 +4642,9 @@
       </c>
       <c r="C252" s="2">
         <v>0.55000000000000004</v>
+      </c>
+      <c r="D252" s="3">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>